<commit_message>
Update new files and remove any redudant
</commit_message>
<xml_diff>
--- a/project-management/stjude-biohackathon-kids26-team15-info.xlsx
+++ b/project-management/stjude-biohackathon-kids26-team15-info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/developmentalneurobiology/core_operations/Bioinformatics/achroni/GitHub/stjude-biohackathon/stjude-biohackathon-KIDS26/KIDS26-Team15/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78AB9ACC-E4C4-414A-91C9-F906AA07EA2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A76DF45-5576-1042-B37D-3F06A71B2A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36180" yWindow="2400" windowWidth="37180" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="280" yWindow="1660" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="team" sheetId="33" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="152">
   <si>
     <t>First Name</t>
   </si>
@@ -400,18 +400,12 @@
     <t>Describe your interest</t>
   </si>
   <si>
-    <t>Lindsey/Rachana</t>
-  </si>
-  <si>
     <t>GitHub PRs/reviews: docs, code</t>
   </si>
   <si>
     <t>I'm applying to the St. Jude BioHackathon because the AI and Data Learning Assistant challenge sits at the intersection of what I do every day and what I care about most: making knowledge findable and helping people build new skills faster. As an Enterprise Architect at International Paper, I design retrieval-augmented generation (RAG) and LLM solutions, help set our AI strategy, and have spent years turning fragmented knowledge platforms into unified, searchable resources. I've also built onboarding tooling and championed best-practice governance — the very problems this project sets out to solve. I hope to contribute hands-on architecture and engineering: designing retrieval pipelines over curated sources like The Turing Way, shaping role-based personalization, and grounding the assistant in accuracy and open-science principles researchers can trust. My span across full-stack development, cloud, and AI lets me move quickly from concept to prototype. In return, I hope to apply my skills somewhere that matters — supporting researchers whose work saves children's lives — while collaborating with data scientists and learning how open-science and reproducibility practices shape real research. I'd be honored to take part.</t>
   </si>
   <si>
-    <t>Rojina/Sarthak Sunil/A. S. M. Tanjim</t>
-  </si>
-  <si>
     <t>testing</t>
   </si>
   <si>
@@ -430,9 +424,6 @@
     <t>I am a final-year undergraduate student with interests in molecular biology, computational biology, and single-cell omics. I enjoy learning new research skills and reading journals online. Through research projects, I have gained experience in single-cell transcriptomic data analysis, bioinformatics tool development, and drug repurposing research. Recently, we have developed a bioinformatics tool for drug repurposing in our computational biology lab.  I am a team person. I enjoy working in a collaborative environment and respect others’ opinions. I have technical expertise in R and Python, shell scripting, automated workflow development, and genomic and transcriptomic data analysis.  In Bangladesh, life science is still a growing sector. We, university students, usually don’t get an opportunity to participate in a biohackathon. Universities don’t get enough funds for research activities. We have brilliant minds, but we graduate with a bare minimum of theoretical knowledge in our domain. My technical skills are mostly self-taught.  KIDS 2026 is a great opportunity to participate in a global event. I am eager to learn from other participants. I want to learn how others approach a scientific problem from their perspective, troubleshoot, and discuss the solution with others. I believe that the collaborative nature of the biohackathon would help me expand my computational biology research opportunities in my home country.</t>
   </si>
   <si>
-    <t>GitHub PRs/reviews: docs</t>
-  </si>
-  <si>
     <t xml:space="preserve">no </t>
   </si>
   <si>
@@ -452,6 +443,57 @@
   </si>
   <si>
     <t>I'm a second-year Honours Biochemistry student at McMaster University working at the intersection of computation and biology. I currently work in Dongdong Wang's computational pathology lab building H&amp;E histology quantification pipelines, and recently completed snRNA-seq analysis identifying gene expression signatures in glioblastoma datasets. I'm also the founder of Sunbeam Health, an AI clinical documentation platform incubated at Harvard's Health Systems Innovation Lab, and built OpenGeneEdit, a fine-tuned LLM with RAG over the iGEM registry for genetic circuit design. My interest in this hackathon is personal. I lost a close family member to cancer young, and that experience drives my commitment to building tools that improve patient outcomes. St. Jude's mission resonates deeply. I'd contribute strong computational and biological skills: comfortable across Python, ML, cloud infrastructure, and genomic data analysis, with experience shipping products under pressure through startup accelerators. I hope to gain exposure to pediatric cancer data science challenges, collaborate with mission-aligned researchers, and bring new methods back to my computational pathology work.</t>
+  </si>
+  <si>
+    <t>Interested in</t>
+  </si>
+  <si>
+    <t>Lindsey/Sarthak</t>
+  </si>
+  <si>
+    <t>setting up the README (deliverable); presentation (slides); learn Rust</t>
+  </si>
+  <si>
+    <t>beginner</t>
+  </si>
+  <si>
+    <t>high (mostly ADO, but transferrable)</t>
+  </si>
+  <si>
+    <t>GitHub Copilot, Claude code, Hermes</t>
+  </si>
+  <si>
+    <t>Automated ROI detection and impact of the project? GitHub PR reviewer</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>moderate</t>
+  </si>
+  <si>
+    <t>Rojina/Antonia</t>
+  </si>
+  <si>
+    <t>Code development and review; HPC testing</t>
+  </si>
+  <si>
+    <t>No (Bangladesh); be available throughout the biohackathon event. Bangladesh standard time is 11 hours ahead of CDT. It's 4 AM here and I am still awake :). I will be available whenever the team needs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">besides the assigned task- presentation(slides), can help with setting README as well. </t>
+  </si>
+  <si>
+    <t>intermediate</t>
+  </si>
+  <si>
+    <t>Rachana/A.S.M. Tanjim</t>
+  </si>
+  <si>
+    <t>Biology of sc-rna</t>
+  </si>
+  <si>
+    <t>Testing results/Biology of sc-rna; GitHub PR reviewer</t>
   </si>
 </sst>
 </file>
@@ -662,7 +704,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -711,6 +753,9 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="5" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -942,11 +987,11 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="2"/>
-    <col min="3" max="3" width="19.5" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="52.5" style="2" customWidth="1"/>
-    <col min="5" max="5" width="18.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="39.1640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="9.6640625" style="2" customWidth="1"/>
-    <col min="7" max="8" width="26.83203125" style="2" customWidth="1"/>
+    <col min="7" max="8" width="17" style="2" customWidth="1"/>
     <col min="9" max="9" width="9.83203125" style="2" customWidth="1"/>
     <col min="10" max="10" width="15.5" style="2" customWidth="1"/>
     <col min="11" max="11" width="20" style="2" customWidth="1"/>
@@ -977,81 +1022,83 @@
         <v>15</v>
       </c>
       <c r="E1" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="M1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="N1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="10" t="s">
+      <c r="O1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="P1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="Q1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="R1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="S1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="T1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="T1" s="11" t="s">
+      <c r="U1" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="V1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="W1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="W1" s="7" t="s">
+      <c r="X1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="X1" s="7" t="s">
+      <c r="Y1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="Z1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="Z1" s="7" t="s">
+      <c r="AA1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="AA1" s="12" t="s">
+      <c r="AB1" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="AB1" s="7" t="s">
+      <c r="AC1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="AC1" s="11" t="s">
+      <c r="AD1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="AD1" s="13"/>
       <c r="AE1" s="13"/>
       <c r="AF1" s="13"/>
       <c r="AG1" s="13"/>
@@ -1069,77 +1116,85 @@
         <v>28</v>
       </c>
       <c r="C2" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="E2" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="J2" s="36" t="s">
+        <v>139</v>
+      </c>
+      <c r="K2" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="L2" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="P2" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q2" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="T2" s="20" t="s">
+        <v>140</v>
+      </c>
+      <c r="U2" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="V2" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="W2" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="X2" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y2" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z2" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB2" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="K2" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="L2" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="M2" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="N2" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q2" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="R2" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="S2" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="T2" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="U2" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="V2" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="W2" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="X2" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y2" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="Z2" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="AA2" s="22" t="s">
-        <v>122</v>
-      </c>
-      <c r="AB2" s="23" t="s">
+      <c r="AC2" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="AC2" s="20" t="s">
+      <c r="AD2" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="AD2" s="16"/>
       <c r="AE2" s="16"/>
       <c r="AF2" s="16"/>
       <c r="AG2" s="16"/>
@@ -1157,75 +1212,85 @@
         <v>41</v>
       </c>
       <c r="C3" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="N3" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="O3" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="P3" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q3" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="R3" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="S3" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="T3" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="V3" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="W3" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="X3" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y3" s="14"/>
+      <c r="Z3" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA3" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB3" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="D3" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="L3" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="M3" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="N3" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="O3" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q3" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="R3" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="S3" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="T3" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="U3" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="V3" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="W3" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="X3" s="14"/>
-      <c r="Y3" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z3" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="AA3" s="22" t="s">
-        <v>125</v>
-      </c>
-      <c r="AB3" s="23" t="s">
+      <c r="AC3" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="AC3" s="20" t="s">
+      <c r="AD3" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="AD3" s="16"/>
       <c r="AE3" s="16"/>
       <c r="AF3" s="16"/>
       <c r="AG3" s="16"/>
@@ -1243,77 +1308,79 @@
         <v>51</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="15"/>
       <c r="G4" s="15"/>
-      <c r="H4" s="17"/>
+      <c r="H4" s="15" t="s">
+        <v>33</v>
+      </c>
       <c r="I4" s="17"/>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="17"/>
+      <c r="K4" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="K4" s="14" t="s">
+      <c r="L4" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="L4" s="18" t="s">
-        <v>33</v>
-      </c>
       <c r="M4" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N4" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="O4" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="O4" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="15" t="s">
-        <v>33</v>
+      <c r="P4" s="18" t="s">
+        <v>31</v>
       </c>
       <c r="Q4" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="R4" s="20" t="s">
+      <c r="R4" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="S4" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="S4" s="20" t="s">
+      <c r="T4" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="T4" s="20" t="s">
-        <v>33</v>
-      </c>
       <c r="U4" s="20" t="s">
         <v>33</v>
       </c>
       <c r="V4" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="W4" s="14" t="s">
+      <c r="W4" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="X4" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="X4" s="14" t="s">
+      <c r="Y4" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="Y4" s="14" t="s">
+      <c r="Z4" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="Z4" s="21" t="s">
+      <c r="AA4" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="AA4" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="AB4" s="23" t="s">
+      <c r="AB4" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="AC4" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="AC4" s="20" t="s">
+      <c r="AD4" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="AD4" s="16"/>
       <c r="AE4" s="16"/>
       <c r="AF4" s="16"/>
       <c r="AG4" s="16"/>
@@ -1331,75 +1398,85 @@
         <v>62</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>123</v>
+        <v>149</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="K5" s="20" t="s">
+      <c r="F5" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="L5" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="L5" s="18" t="s">
-        <v>31</v>
-      </c>
       <c r="M5" s="18" t="s">
         <v>31</v>
       </c>
       <c r="N5" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="O5" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="O5" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="15" t="s">
-        <v>33</v>
+      <c r="P5" s="18" t="s">
+        <v>31</v>
       </c>
       <c r="Q5" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="R5" s="20" t="s">
+      <c r="R5" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="S5" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="S5" s="20" t="s">
+      <c r="T5" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="T5" s="20" t="s">
-        <v>33</v>
-      </c>
       <c r="U5" s="20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="V5" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="W5" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="W5" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="X5" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="X5" s="14"/>
-      <c r="Y5" s="14" t="s">
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="Z5" s="21" t="s">
+      <c r="AA5" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="AA5" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="AB5" s="23" t="s">
+      <c r="AB5" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="AC5" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="AC5" s="20" t="s">
+      <c r="AD5" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="AD5" s="16"/>
       <c r="AE5" s="16"/>
       <c r="AF5" s="16"/>
       <c r="AG5" s="16"/>
@@ -1417,77 +1494,87 @@
         <v>70</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
+        <v>151</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>33</v>
+      </c>
       <c r="G6" s="15"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="14" t="s">
+      <c r="H6" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="K6" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="K6" s="14" t="s">
+      <c r="L6" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="L6" s="18" t="s">
-        <v>31</v>
-      </c>
       <c r="M6" s="18" t="s">
         <v>31</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>131</v>
+        <v>31</v>
       </c>
       <c r="O6" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="P6" s="15" t="s">
-        <v>33</v>
+        <v>128</v>
+      </c>
+      <c r="P6" s="18" t="s">
+        <v>31</v>
       </c>
       <c r="Q6" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="R6" s="20" t="s">
+      <c r="R6" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="S6" s="20" t="s">
+      <c r="T6" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="T6" s="20" t="s">
-        <v>33</v>
-      </c>
       <c r="U6" s="20" t="s">
         <v>33</v>
       </c>
       <c r="V6" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="W6" s="14" t="s">
+      <c r="W6" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="X6" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="X6" s="14" t="s">
+      <c r="Y6" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="Y6" s="14" t="s">
+      <c r="Z6" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="Z6" s="21" t="s">
+      <c r="AA6" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="AA6" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="AB6" s="23" t="s">
+      <c r="AB6" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="AC6" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="AC6" s="24" t="s">
+      <c r="AD6" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="AD6" s="16"/>
       <c r="AE6" s="16"/>
       <c r="AF6" s="16"/>
       <c r="AG6" s="16"/>
@@ -1506,80 +1593,80 @@
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
-      <c r="E7" s="15" t="s">
-        <v>33</v>
-      </c>
+      <c r="E7" s="15"/>
       <c r="F7" s="15" t="s">
         <v>33</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="H7" s="17" t="s">
-        <v>133</v>
+      <c r="H7" s="15" t="s">
+        <v>33</v>
       </c>
       <c r="I7" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="J7" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="J7" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="K7" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="K7" s="14" t="s">
+      <c r="L7" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="L7" s="18" t="s">
-        <v>31</v>
-      </c>
       <c r="M7" s="18" t="s">
         <v>31</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="O7" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="P7" s="15" t="s">
+      <c r="P7" s="18" t="s">
         <v>33</v>
       </c>
       <c r="Q7" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="R7" s="20" t="s">
-        <v>31</v>
+      <c r="R7" s="15" t="s">
+        <v>33</v>
       </c>
       <c r="S7" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="T7" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="T7" s="20" t="s">
-        <v>33</v>
-      </c>
       <c r="U7" s="20" t="s">
         <v>33</v>
       </c>
       <c r="V7" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="W7" s="14"/>
-      <c r="X7" s="14" t="s">
+      <c r="W7" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="Y7" s="14" t="s">
+      <c r="Z7" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="Z7" s="21" t="s">
+      <c r="AA7" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="AA7" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="AB7" s="23" t="s">
+      <c r="AB7" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC7" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="AC7" s="20" t="s">
+      <c r="AD7" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="AD7" s="16"/>
       <c r="AE7" s="16"/>
       <c r="AF7" s="16"/>
       <c r="AG7" s="16"/>
@@ -2441,12 +2528,12 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="AB2" r:id="rId1" display="mailto:lrwarren94@gmail.com" xr:uid="{B8FB5B30-D542-274A-91EE-2FA462363255}"/>
-    <hyperlink ref="AB3" r:id="rId2" display="mailto:sar3142168@gmail.com" xr:uid="{0C958BF8-58A0-764B-B4CA-9DD080E5B670}"/>
-    <hyperlink ref="AB4" r:id="rId3" display="mailto:rsapkota@stjude.org" xr:uid="{2865EBF1-2E3F-614B-8F18-40C48DAB40AA}"/>
-    <hyperlink ref="AB5" r:id="rId4" display="mailto:asmtanjimhassan@gmail.com" xr:uid="{412CDB77-98AB-644B-9CB3-F1C99646D69D}"/>
-    <hyperlink ref="AB6" r:id="rId5" display="mailto:pande250@umn.edu" xr:uid="{E4FD3264-40B2-B647-91F1-34B9DC6AB9D0}"/>
-    <hyperlink ref="AB7" r:id="rId6" display="mailto:antonia.chroni@stjude.org" xr:uid="{F00A6F6E-0674-0941-9930-779FB43A4F20}"/>
+    <hyperlink ref="AC2" r:id="rId1" display="mailto:lrwarren94@gmail.com" xr:uid="{B5569C76-0407-C548-85AB-0E87A151DB53}"/>
+    <hyperlink ref="AC3" r:id="rId2" display="mailto:sar3142168@gmail.com" xr:uid="{E2B400C6-AD2A-314D-A83F-F9280BF2A141}"/>
+    <hyperlink ref="AC4" r:id="rId3" display="mailto:rsapkota@stjude.org" xr:uid="{E7F511B2-3DB3-D042-AD73-A2A2D4300C6F}"/>
+    <hyperlink ref="AC5" r:id="rId4" display="mailto:asmtanjimhassan@gmail.com" xr:uid="{3F3791A1-983D-7B4F-A7A7-3258C3959E46}"/>
+    <hyperlink ref="AC6" r:id="rId5" display="mailto:pande250@umn.edu" xr:uid="{D18E3AD3-23FA-F045-B9CE-04656901CA1B}"/>
+    <hyperlink ref="AC7" r:id="rId6" display="mailto:antonia.chroni@stjude.org" xr:uid="{1E28BF78-2346-D648-ADBD-DD2990204859}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -2537,7 +2624,7 @@
   <sheetData>
     <row r="1" spans="1:30" ht="14" x14ac:dyDescent="0.15">
       <c r="A1" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
@@ -2621,7 +2708,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>87</v>
@@ -2678,7 +2765,7 @@
         <v>38</v>
       </c>
       <c r="V2" s="22" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="W2" s="23" t="s">
         <v>39</v>
@@ -2699,7 +2786,7 @@
         <v>41</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>86</v>
@@ -2754,7 +2841,7 @@
         <v>48</v>
       </c>
       <c r="V3" s="22" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="W3" s="23" t="s">
         <v>49</v>
@@ -2775,7 +2862,7 @@
         <v>51</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>87</v>
@@ -2832,7 +2919,7 @@
         <v>59</v>
       </c>
       <c r="V4" s="22" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="W4" s="23" t="s">
         <v>60</v>
@@ -2853,7 +2940,7 @@
         <v>62</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>86</v>
@@ -2908,7 +2995,7 @@
         <v>67</v>
       </c>
       <c r="V5" s="22" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="W5" s="23" t="s">
         <v>68</v>
@@ -2929,7 +3016,7 @@
         <v>70</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>87</v>
@@ -2947,7 +3034,7 @@
         <v>31</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="J6" s="20" t="s">
         <v>31</v>
@@ -2986,7 +3073,7 @@
         <v>75</v>
       </c>
       <c r="V6" s="22" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="W6" s="23" t="s">
         <v>76</v>
@@ -3007,7 +3094,7 @@
         <v>78</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>87</v>
@@ -3140,7 +3227,7 @@
         <v>59</v>
       </c>
       <c r="V8" s="22" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="W8" s="23" t="s">
         <v>93</v>
@@ -3188,7 +3275,7 @@
         <v>25</v>
       </c>
       <c r="V9" s="33" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="W9" s="34" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Update file sin docs and proejct management
</commit_message>
<xml_diff>
--- a/project-management/stjude-biohackathon-kids26-team15-info.xlsx
+++ b/project-management/stjude-biohackathon-kids26-team15-info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/developmentalneurobiology/core_operations/Bioinformatics/achroni/GitHub/stjude-biohackathon/stjude-biohackathon-KIDS26/KIDS26-Team15/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A76DF45-5576-1042-B37D-3F06A71B2A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C1C1E68-EC42-4F42-B957-A0186CAFC826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="280" yWindow="1660" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1660" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="team" sheetId="33" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="157">
   <si>
     <t>First Name</t>
   </si>
@@ -494,6 +494,21 @@
   </si>
   <si>
     <t>Testing results/Biology of sc-rna; GitHub PR reviewer</t>
+  </si>
+  <si>
+    <t>Emma</t>
+  </si>
+  <si>
+    <t>Bishop</t>
+  </si>
+  <si>
+    <t>Emma/Rojina</t>
+  </si>
+  <si>
+    <t>Code development and review</t>
+  </si>
+  <si>
+    <t>emjbishop</t>
   </si>
 </sst>
 </file>
@@ -983,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D102A30C-A89E-9547-97A0-7BF5921F82B3}">
-  <dimension ref="A1:AL28"/>
+  <dimension ref="A1:AL29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="2"/>
@@ -1000,7 +1015,7 @@
     <col min="14" max="14" width="14.33203125" style="2" customWidth="1"/>
     <col min="15" max="15" width="14" style="2" customWidth="1"/>
     <col min="16" max="16" width="18.33203125" style="2" customWidth="1"/>
-    <col min="17" max="17" width="47.5" style="2" customWidth="1"/>
+    <col min="17" max="17" width="9.33203125" style="2" customWidth="1"/>
     <col min="18" max="18" width="42.33203125" style="2" customWidth="1"/>
     <col min="19" max="19" width="25.83203125" style="2" customWidth="1"/>
     <col min="20" max="20" width="26.1640625" style="2" customWidth="1"/>
@@ -1584,48 +1599,42 @@
       <c r="AK6" s="16"/>
       <c r="AL6" s="16"/>
     </row>
-    <row r="7" spans="1:38" ht="14" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:38" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
-        <v>88</v>
+        <v>152</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
+        <v>153</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>155</v>
+      </c>
       <c r="E7" s="15"/>
-      <c r="F7" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="H7" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="I7" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="J7" s="17" t="s">
-        <v>130</v>
-      </c>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
       <c r="K7" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>90</v>
+        <v>156</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O7" s="18" t="s">
         <v>33</v>
       </c>
       <c r="P7" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="Q7" s="15" t="s">
         <v>33</v>
@@ -1633,40 +1642,18 @@
       <c r="R7" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="S7" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="T7" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="U7" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="V7" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="W7" s="20" t="s">
-        <v>33</v>
-      </c>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="20"/>
       <c r="X7" s="14"/>
-      <c r="Y7" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="Z7" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="AA7" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB7" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="AC7" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="AD7" s="20" t="s">
-        <v>30</v>
-      </c>
+      <c r="Y7" s="14"/>
+      <c r="Z7" s="14"/>
+      <c r="AA7" s="21"/>
+      <c r="AB7" s="22"/>
+      <c r="AC7" s="23"/>
+      <c r="AD7" s="24"/>
       <c r="AE7" s="16"/>
       <c r="AF7" s="16"/>
       <c r="AG7" s="16"/>
@@ -1677,36 +1664,88 @@
       <c r="AL7" s="16"/>
     </row>
     <row r="8" spans="1:38" ht="14" x14ac:dyDescent="0.15">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="16"/>
-      <c r="U8" s="16"/>
-      <c r="V8" s="16"/>
-      <c r="W8" s="16"/>
-      <c r="X8" s="16"/>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="16"/>
-      <c r="AA8" s="16"/>
-      <c r="AB8" s="16"/>
-      <c r="AC8" s="16"/>
-      <c r="AD8" s="16"/>
+      <c r="A8" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="L8" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="M8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="N8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="O8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="P8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q8" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="R8" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="S8" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="T8" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="U8" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="V8" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="W8" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="X8" s="14"/>
+      <c r="Y8" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z8" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="AA8" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB8" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC8" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="AD8" s="20" t="s">
+        <v>30</v>
+      </c>
       <c r="AE8" s="16"/>
       <c r="AF8" s="16"/>
       <c r="AG8" s="16"/>
@@ -1716,7 +1755,7 @@
       <c r="AK8" s="16"/>
       <c r="AL8" s="16"/>
     </row>
-    <row r="9" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:38" ht="14" x14ac:dyDescent="0.15">
       <c r="A9" s="16"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
@@ -1876,7 +1915,7 @@
       <c r="AK12" s="16"/>
       <c r="AL12" s="16"/>
     </row>
-    <row r="13" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="16"/>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -1905,9 +1944,7 @@
       <c r="Z13" s="16"/>
       <c r="AA13" s="16"/>
       <c r="AB13" s="16"/>
-      <c r="AC13" s="27" t="s">
-        <v>3</v>
-      </c>
+      <c r="AC13" s="16"/>
       <c r="AD13" s="16"/>
       <c r="AE13" s="16"/>
       <c r="AF13" s="16"/>
@@ -1918,7 +1955,7 @@
       <c r="AK13" s="16"/>
       <c r="AL13" s="16"/>
     </row>
-    <row r="14" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="16"/>
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
@@ -1947,8 +1984,8 @@
       <c r="Z14" s="16"/>
       <c r="AA14" s="16"/>
       <c r="AB14" s="16"/>
-      <c r="AC14" s="28" t="s">
-        <v>94</v>
+      <c r="AC14" s="27" t="s">
+        <v>3</v>
       </c>
       <c r="AD14" s="16"/>
       <c r="AE14" s="16"/>
@@ -1990,7 +2027,7 @@
       <c r="AA15" s="16"/>
       <c r="AB15" s="16"/>
       <c r="AC15" s="28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AD15" s="16"/>
       <c r="AE15" s="16"/>
@@ -2031,7 +2068,9 @@
       <c r="Z16" s="16"/>
       <c r="AA16" s="16"/>
       <c r="AB16" s="16"/>
-      <c r="AC16" s="16"/>
+      <c r="AC16" s="28" t="s">
+        <v>95</v>
+      </c>
       <c r="AD16" s="16"/>
       <c r="AE16" s="16"/>
       <c r="AF16" s="16"/>
@@ -2071,9 +2110,7 @@
       <c r="Z17" s="16"/>
       <c r="AA17" s="16"/>
       <c r="AB17" s="16"/>
-      <c r="AC17" s="29" t="s">
-        <v>96</v>
-      </c>
+      <c r="AC17" s="16"/>
       <c r="AD17" s="16"/>
       <c r="AE17" s="16"/>
       <c r="AF17" s="16"/>
@@ -2114,7 +2151,7 @@
       <c r="AA18" s="16"/>
       <c r="AB18" s="16"/>
       <c r="AC18" s="29" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AD18" s="16"/>
       <c r="AE18" s="16"/>
@@ -2155,7 +2192,9 @@
       <c r="Z19" s="16"/>
       <c r="AA19" s="16"/>
       <c r="AB19" s="16"/>
-      <c r="AC19" s="16"/>
+      <c r="AC19" s="29" t="s">
+        <v>97</v>
+      </c>
       <c r="AD19" s="16"/>
       <c r="AE19" s="16"/>
       <c r="AF19" s="16"/>
@@ -2406,7 +2445,7 @@
       <c r="AK25" s="16"/>
       <c r="AL25" s="16"/>
     </row>
-    <row r="26" spans="1:38" ht="14" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:38" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
@@ -2526,6 +2565,46 @@
       <c r="AK28" s="16"/>
       <c r="AL28" s="16"/>
     </row>
+    <row r="29" spans="1:38" ht="14" x14ac:dyDescent="0.15">
+      <c r="A29" s="16"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="16"/>
+      <c r="N29" s="16"/>
+      <c r="O29" s="16"/>
+      <c r="P29" s="16"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="16"/>
+      <c r="S29" s="16"/>
+      <c r="T29" s="16"/>
+      <c r="U29" s="16"/>
+      <c r="V29" s="16"/>
+      <c r="W29" s="16"/>
+      <c r="X29" s="16"/>
+      <c r="Y29" s="16"/>
+      <c r="Z29" s="16"/>
+      <c r="AA29" s="16"/>
+      <c r="AB29" s="16"/>
+      <c r="AC29" s="16"/>
+      <c r="AD29" s="16"/>
+      <c r="AE29" s="16"/>
+      <c r="AF29" s="16"/>
+      <c r="AG29" s="16"/>
+      <c r="AH29" s="16"/>
+      <c r="AI29" s="16"/>
+      <c r="AJ29" s="16"/>
+      <c r="AK29" s="16"/>
+      <c r="AL29" s="16"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="AC2" r:id="rId1" display="mailto:lrwarren94@gmail.com" xr:uid="{B5569C76-0407-C548-85AB-0E87A151DB53}"/>
@@ -2533,7 +2612,7 @@
     <hyperlink ref="AC4" r:id="rId3" display="mailto:rsapkota@stjude.org" xr:uid="{E7F511B2-3DB3-D042-AD73-A2A2D4300C6F}"/>
     <hyperlink ref="AC5" r:id="rId4" display="mailto:asmtanjimhassan@gmail.com" xr:uid="{3F3791A1-983D-7B4F-A7A7-3258C3959E46}"/>
     <hyperlink ref="AC6" r:id="rId5" display="mailto:pande250@umn.edu" xr:uid="{D18E3AD3-23FA-F045-B9CE-04656901CA1B}"/>
-    <hyperlink ref="AC7" r:id="rId6" display="mailto:antonia.chroni@stjude.org" xr:uid="{1E28BF78-2346-D648-ADBD-DD2990204859}"/>
+    <hyperlink ref="AC8" r:id="rId6" display="mailto:antonia.chroni@stjude.org" xr:uid="{1E28BF78-2346-D648-ADBD-DD2990204859}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>